<commit_message>
Update 25MMS5504-NIIT-CISCO-US-Attendance Roster_Splunk Intermediate_9-11 Mar'26.xlsx
</commit_message>
<xml_diff>
--- a/25MMS5504-NIIT-CISCO-US-Attendance Roster_Splunk Intermediate_9-11 Mar'26.xlsx
+++ b/25MMS5504-NIIT-CISCO-US-Attendance Roster_Splunk Intermediate_9-11 Mar'26.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Vivek\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\VK_GIT\CISCO_US_09_03_2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1AF3086F-9D56-49EB-A252-DE6F130E13FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F49FC9A5-F57E-4BBF-A6CE-89CAAD8045FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -187,7 +187,7 @@
     <t>Password</t>
   </si>
   <si>
-    <t>URL - https://cloud.rpsconsulting.in/console/#/</t>
+    <t>URL - https://cloud.cdp.rpsconsulting.in/console</t>
   </si>
 </sst>
 </file>
@@ -634,6 +634,45 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="19" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="20" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="20" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
@@ -642,45 +681,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="19" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="20" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="20" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -974,11 +974,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B1" s="29" t="s">
+      <c r="B1" s="42" t="s">
         <v>8</v>
       </c>
-      <c r="C1" s="30"/>
-      <c r="D1" s="31"/>
+      <c r="C1" s="43"/>
+      <c r="D1" s="44"/>
     </row>
     <row r="2" spans="1:5" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
@@ -1239,207 +1239,207 @@
       </c>
     </row>
     <row r="10" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B10" s="38" t="s">
+      <c r="B10" s="35" t="s">
         <v>5</v>
       </c>
-      <c r="C10" s="38" t="s">
+      <c r="C10" s="35" t="s">
         <v>6</v>
       </c>
-      <c r="D10" s="38" t="s">
+      <c r="D10" s="35" t="s">
         <v>48</v>
       </c>
-      <c r="E10" s="38" t="s">
+      <c r="E10" s="35" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="11" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B11" s="39" t="s">
+      <c r="B11" s="36" t="s">
         <v>20</v>
       </c>
-      <c r="C11" s="40" t="s">
+      <c r="C11" s="37" t="s">
         <v>32</v>
       </c>
-      <c r="D11" s="41" t="s">
+      <c r="D11" s="38" t="s">
         <v>34</v>
       </c>
-      <c r="E11" s="42" t="s">
+      <c r="E11" s="39" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="12" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B12" s="39" t="s">
+      <c r="B12" s="36" t="s">
         <v>19</v>
       </c>
-      <c r="C12" s="40" t="s">
+      <c r="C12" s="37" t="s">
         <v>31</v>
       </c>
-      <c r="D12" s="41" t="s">
+      <c r="D12" s="38" t="s">
         <v>36</v>
       </c>
-      <c r="E12" s="42" t="s">
+      <c r="E12" s="39" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="13" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B13" s="39" t="s">
+      <c r="B13" s="36" t="s">
         <v>13</v>
       </c>
-      <c r="C13" s="40" t="s">
+      <c r="C13" s="37" t="s">
         <v>25</v>
       </c>
-      <c r="D13" s="41" t="s">
+      <c r="D13" s="38" t="s">
         <v>37</v>
       </c>
-      <c r="E13" s="43" t="s">
+      <c r="E13" s="40" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="14" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B14" s="44" t="s">
+      <c r="B14" s="41" t="s">
         <v>12</v>
       </c>
-      <c r="C14" s="40" t="s">
+      <c r="C14" s="37" t="s">
         <v>24</v>
       </c>
-      <c r="D14" s="41" t="s">
+      <c r="D14" s="38" t="s">
         <v>38</v>
       </c>
-      <c r="E14" s="43" t="s">
+      <c r="E14" s="40" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="15" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B15" s="39" t="s">
+      <c r="B15" s="36" t="s">
         <v>18</v>
       </c>
-      <c r="C15" s="40" t="s">
+      <c r="C15" s="37" t="s">
         <v>30</v>
       </c>
-      <c r="D15" s="41" t="s">
+      <c r="D15" s="38" t="s">
         <v>39</v>
       </c>
-      <c r="E15" s="42" t="s">
+      <c r="E15" s="39" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="16" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B16" s="39" t="s">
+      <c r="B16" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="C16" s="40" t="s">
+      <c r="C16" s="37" t="s">
         <v>29</v>
       </c>
-      <c r="D16" s="41" t="s">
+      <c r="D16" s="38" t="s">
         <v>40</v>
       </c>
-      <c r="E16" s="42" t="s">
+      <c r="E16" s="39" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="17" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B17" s="39" t="s">
+      <c r="B17" s="36" t="s">
         <v>16</v>
       </c>
-      <c r="C17" s="40" t="s">
+      <c r="C17" s="37" t="s">
         <v>28</v>
       </c>
-      <c r="D17" s="41" t="s">
+      <c r="D17" s="38" t="s">
         <v>41</v>
       </c>
-      <c r="E17" s="43" t="s">
+      <c r="E17" s="40" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="18" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B18" s="39" t="s">
+      <c r="B18" s="36" t="s">
         <v>14</v>
       </c>
-      <c r="C18" s="40" t="s">
+      <c r="C18" s="37" t="s">
         <v>26</v>
       </c>
-      <c r="D18" s="41" t="s">
+      <c r="D18" s="38" t="s">
         <v>42</v>
       </c>
-      <c r="E18" s="42" t="s">
+      <c r="E18" s="39" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="19" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B19" s="39" t="s">
+      <c r="B19" s="36" t="s">
         <v>11</v>
       </c>
-      <c r="C19" s="40" t="s">
+      <c r="C19" s="37" t="s">
         <v>23</v>
       </c>
-      <c r="D19" s="41" t="s">
+      <c r="D19" s="38" t="s">
         <v>43</v>
       </c>
-      <c r="E19" s="42" t="s">
+      <c r="E19" s="39" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="20" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B20" s="39" t="s">
+      <c r="B20" s="36" t="s">
         <v>10</v>
       </c>
-      <c r="C20" s="40" t="s">
+      <c r="C20" s="37" t="s">
         <v>22</v>
       </c>
-      <c r="D20" s="41" t="s">
+      <c r="D20" s="38" t="s">
         <v>44</v>
       </c>
-      <c r="E20" s="42" t="s">
+      <c r="E20" s="39" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="21" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B21" s="39" t="s">
+      <c r="B21" s="36" t="s">
         <v>15</v>
       </c>
-      <c r="C21" s="40" t="s">
+      <c r="C21" s="37" t="s">
         <v>27</v>
       </c>
-      <c r="D21" s="41" t="s">
+      <c r="D21" s="38" t="s">
         <v>45</v>
       </c>
-      <c r="E21" s="42" t="s">
+      <c r="E21" s="39" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="22" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B22" s="39" t="s">
+      <c r="B22" s="36" t="s">
         <v>21</v>
       </c>
-      <c r="C22" s="40" t="s">
+      <c r="C22" s="37" t="s">
         <v>33</v>
       </c>
-      <c r="D22" s="41" t="s">
+      <c r="D22" s="38" t="s">
         <v>46</v>
       </c>
-      <c r="E22" s="43" t="s">
+      <c r="E22" s="40" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="23" spans="2:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B23" s="36"/>
-      <c r="C23" s="37"/>
-      <c r="D23" s="33"/>
-      <c r="E23" s="35"/>
+      <c r="B23" s="33"/>
+      <c r="C23" s="34"/>
+      <c r="D23" s="30"/>
+      <c r="E23" s="32"/>
     </row>
     <row r="24" spans="2:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B24" s="36"/>
-      <c r="C24" s="37"/>
-      <c r="D24" s="33"/>
-      <c r="E24" s="35"/>
+      <c r="B24" s="33"/>
+      <c r="C24" s="34"/>
+      <c r="D24" s="30"/>
+      <c r="E24" s="32"/>
     </row>
     <row r="25" spans="2:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="D25" s="32">
+      <c r="D25" s="29">
         <v>13</v>
       </c>
-      <c r="E25" s="33" t="s">
+      <c r="E25" s="30" t="s">
         <v>47</v>
       </c>
-      <c r="F25" s="34" t="s">
+      <c r="F25" s="31" t="s">
         <v>35</v>
       </c>
     </row>

</xml_diff>